<commit_message>
update CNC_Pen-ploter.xlsx and remove temporary file
</commit_message>
<xml_diff>
--- a/BOM/CNC_Pen-ploter.xlsx
+++ b/BOM/CNC_Pen-ploter.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nitin\Documents\.Glyph-Writer\CNC-pen-ploter\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5ECBCCD0-2931-445D-A6CE-788A0258057D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDF2312-6DB9-4567-9845-678C01013EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="rId1"/>

</xml_diff>